<commit_message>
Variante 3ch: PCB didattico rifatto a blocchi, test point accanto ai nodi
- piazzamento a fasce: alimentazione, 3 canali identici (segnale in alto
  da sinistra a destra, circuiti di supporto sotto), coincidenza in basso
- test point a pochi mm dal nodo misurato (SIG_IN 94 -> 9 mm di pista)
- uscite verso la coincidenza in un corridoio riservato sul bordo destro
- serigrafia didattica (silk3.py): blocchi numerati, titoli, etichette dei
  test point e dei connettori, riferimenti, schema a blocchi, legenda
  'Come funziona' sul retro; identica in KiCad (gr_poly) e nei Gerber
- ingressi dell'AND riassegnati (equivalenti) per piste senza incroci
- Keystone 5000 rosso / 5001 nero anche nella BOM

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fc9yPsNewCQrMK8R1c8Ls
</commit_message>
<xml_diff>
--- a/hardware/variante_3ch/jlcpcb/CPL_JLCPCB.xlsx
+++ b/hardware/variante_3ch/jlcpcb/CPL_JLCPCB.xlsx
@@ -451,12 +451,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>14.000mm</t>
+          <t>39.000mm</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>131.000mm</t>
+          <t>188.500mm</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -478,12 +478,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20.000mm</t>
+          <t>44.500mm</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>140.500mm</t>
+          <t>198.000mm</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -505,12 +505,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>24.000mm</t>
+          <t>48.500mm</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>140.500mm</t>
+          <t>198.000mm</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -532,12 +532,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4.000mm</t>
+          <t>29.000mm</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>144.000mm</t>
+          <t>201.000mm</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -559,12 +559,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>24.500mm</t>
+          <t>10.500mm</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>117.000mm</t>
+          <t>132.000mm</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -586,12 +586,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>14.500mm</t>
+          <t>12.000mm</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>148.000mm</t>
+          <t>156.500mm</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -613,12 +613,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.500mm</t>
+          <t>16.500mm</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>156.000mm</t>
+          <t>164.000mm</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -640,12 +640,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>51.500mm</t>
+          <t>54.500mm</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>148.500mm</t>
+          <t>156.500mm</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -667,12 +667,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>40.500mm</t>
+          <t>43.500mm</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>156.000mm</t>
+          <t>164.000mm</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -694,12 +694,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>58.000mm</t>
+          <t>65.000mm</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>141.000mm</t>
+          <t>136.000mm</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -721,12 +721,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>24.500mm</t>
+          <t>10.500mm</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>62.000mm</t>
+          <t>80.000mm</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -748,12 +748,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14.500mm</t>
+          <t>12.000mm</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>93.000mm</t>
+          <t>104.500mm</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -775,12 +775,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>13.500mm</t>
+          <t>16.500mm</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>101.000mm</t>
+          <t>112.000mm</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -802,12 +802,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>51.500mm</t>
+          <t>54.500mm</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>93.500mm</t>
+          <t>104.500mm</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -829,12 +829,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>40.500mm</t>
+          <t>43.500mm</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>101.000mm</t>
+          <t>112.000mm</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -856,12 +856,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>58.000mm</t>
+          <t>65.000mm</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>86.000mm</t>
+          <t>84.000mm</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -883,12 +883,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>24.500mm</t>
+          <t>10.500mm</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>7.000mm</t>
+          <t>28.000mm</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -910,12 +910,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>14.500mm</t>
+          <t>12.000mm</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>38.000mm</t>
+          <t>52.500mm</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -937,12 +937,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>13.500mm</t>
+          <t>16.500mm</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>46.000mm</t>
+          <t>60.000mm</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -964,12 +964,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>51.500mm</t>
+          <t>54.500mm</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>38.500mm</t>
+          <t>52.500mm</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -991,12 +991,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>40.500mm</t>
+          <t>43.500mm</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>46.000mm</t>
+          <t>60.000mm</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1018,12 +1018,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>58.000mm</t>
+          <t>65.000mm</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>31.000mm</t>
+          <t>32.000mm</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1045,12 +1045,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>60.600mm</t>
+          <t>67.000mm</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>137.200mm</t>
+          <t>197.000mm</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1072,12 +1072,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>41.500mm</t>
+          <t>67.000mm</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>127.500mm</t>
+          <t>187.000mm</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -1099,12 +1099,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>72.300mm</t>
+          <t>14.000mm</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>124.200mm</t>
+          <t>185.000mm</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1126,12 +1126,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>60.000mm</t>
+          <t>20.000mm</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>123.500mm</t>
+          <t>185.000mm</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1153,12 +1153,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>66.500mm</t>
+          <t>82.000mm</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>69.500mm</t>
+          <t>14.500mm</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1180,12 +1180,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>24.500mm</t>
+          <t>27.500mm</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>163.500mm</t>
+          <t>171.500mm</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1207,12 +1207,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>51.500mm</t>
+          <t>54.500mm</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>161.000mm</t>
+          <t>169.000mm</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1234,12 +1234,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>69.000mm</t>
+          <t>76.000mm</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>150.000mm</t>
+          <t>145.000mm</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1261,12 +1261,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>58.500mm</t>
+          <t>65.500mm</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>145.000mm</t>
+          <t>140.000mm</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1288,12 +1288,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>64.500mm</t>
+          <t>73.000mm</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>132.500mm</t>
+          <t>170.000mm</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1315,12 +1315,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>24.500mm</t>
+          <t>27.500mm</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>108.500mm</t>
+          <t>119.500mm</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1342,12 +1342,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>51.500mm</t>
+          <t>54.500mm</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>106.000mm</t>
+          <t>117.000mm</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1369,12 +1369,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>69.000mm</t>
+          <t>76.000mm</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>95.000mm</t>
+          <t>93.000mm</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>58.500mm</t>
+          <t>65.500mm</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>90.000mm</t>
+          <t>88.000mm</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1423,12 +1423,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>64.500mm</t>
+          <t>73.000mm</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>77.500mm</t>
+          <t>118.000mm</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1450,12 +1450,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>24.500mm</t>
+          <t>27.500mm</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>53.500mm</t>
+          <t>67.500mm</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1477,12 +1477,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>51.500mm</t>
+          <t>54.500mm</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>51.000mm</t>
+          <t>65.000mm</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1504,12 +1504,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>69.000mm</t>
+          <t>76.000mm</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>40.000mm</t>
+          <t>41.000mm</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>58.500mm</t>
+          <t>65.500mm</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>35.000mm</t>
+          <t>36.000mm</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>64.500mm</t>
+          <t>73.000mm</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>22.500mm</t>
+          <t>66.000mm</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1585,12 +1585,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>72.500mm</t>
+          <t>79.500mm</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>139.000mm</t>
+          <t>134.000mm</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1612,12 +1612,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>72.500mm</t>
+          <t>79.500mm</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>84.000mm</t>
+          <t>82.000mm</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1639,12 +1639,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>72.500mm</t>
+          <t>79.500mm</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>29.000mm</t>
+          <t>30.000mm</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1666,12 +1666,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>7.000mm</t>
+          <t>31.000mm</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>137.500mm</t>
+          <t>194.000mm</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1693,12 +1693,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>22.000mm</t>
+          <t>25.000mm</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>154.117mm</t>
+          <t>162.117mm</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1720,12 +1720,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>32.500mm</t>
+          <t>35.500mm</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>155.383mm</t>
+          <t>163.383mm</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1747,12 +1747,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>22.000mm</t>
+          <t>25.000mm</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>99.117mm</t>
+          <t>110.117mm</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1774,12 +1774,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>32.500mm</t>
+          <t>35.500mm</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>100.383mm</t>
+          <t>111.383mm</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1801,12 +1801,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>22.000mm</t>
+          <t>25.000mm</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>44.117mm</t>
+          <t>58.117mm</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1828,12 +1828,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>32.500mm</t>
+          <t>35.500mm</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>45.383mm</t>
+          <t>59.383mm</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>4.000mm</t>
+          <t>49.500mm</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>121.000mm</t>
+          <t>188.000mm</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -1882,12 +1882,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>4.000mm</t>
+          <t>46.500mm</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>124.000mm</t>
+          <t>188.000mm</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -1909,12 +1909,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>14.000mm</t>
+          <t>39.000mm</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>134.000mm</t>
+          <t>192.000mm</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1936,12 +1936,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>4.000mm</t>
+          <t>43.500mm</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>127.000mm</t>
+          <t>188.000mm</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -1963,12 +1963,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>69.500mm</t>
+          <t>85.500mm</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>66.000mm</t>
+          <t>8.500mm</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
     </row>
@@ -1990,12 +1990,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>58.000mm</t>
+          <t>61.200mm</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>64.500mm</t>
+          <t>13.000mm</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
@@ -2017,12 +2017,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>60.000mm</t>
+          <t>67.200mm</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>64.500mm</t>
+          <t>13.000mm</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
@@ -2044,12 +2044,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>61.500mm</t>
+          <t>73.200mm</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>69.500mm</t>
+          <t>13.000mm</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
@@ -2071,12 +2071,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>21.000mm</t>
+          <t>7.000mm</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>128.500mm</t>
+          <t>143.500mm</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2098,12 +2098,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>27.000mm</t>
+          <t>13.000mm</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>130.000mm</t>
+          <t>145.000mm</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2125,12 +2125,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>21.500mm</t>
+          <t>7.500mm</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>120.500mm</t>
+          <t>135.500mm</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2152,12 +2152,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>26.000mm</t>
+          <t>12.000mm</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>113.500mm</t>
+          <t>128.500mm</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>148.000mm</t>
+          <t>156.500mm</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -2206,12 +2206,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>17.000mm</t>
+          <t>20.000mm</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>151.500mm</t>
+          <t>159.500mm</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2233,12 +2233,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>10.000mm</t>
+          <t>11.500mm</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>151.500mm</t>
+          <t>163.000mm</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
@@ -2260,12 +2260,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>22.000mm</t>
+          <t>25.000mm</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>160.500mm</t>
+          <t>168.500mm</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2287,12 +2287,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>28.000mm</t>
+          <t>31.000mm</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>160.500mm</t>
+          <t>168.500mm</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2314,12 +2314,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>32.500mm</t>
+          <t>35.500mm</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>160.500mm</t>
+          <t>168.500mm</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2341,12 +2341,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>36.500mm</t>
+          <t>39.500mm</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>151.500mm</t>
+          <t>159.500mm</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2368,12 +2368,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>44.000mm</t>
+          <t>47.000mm</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>151.500mm</t>
+          <t>159.500mm</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2395,12 +2395,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>46.500mm</t>
+          <t>49.500mm</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>148.500mm</t>
+          <t>156.500mm</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2422,12 +2422,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>46.000mm</t>
+          <t>49.000mm</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>144.000mm</t>
+          <t>152.000mm</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2449,12 +2449,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>36.000mm</t>
+          <t>39.000mm</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>139.000mm</t>
+          <t>143.500mm</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2476,12 +2476,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>49.000mm</t>
+          <t>52.000mm</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>138.500mm</t>
+          <t>143.000mm</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2503,12 +2503,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>58.000mm</t>
+          <t>65.000mm</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>149.500mm</t>
+          <t>144.500mm</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2530,12 +2530,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>72.500mm</t>
+          <t>79.500mm</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>145.000mm</t>
+          <t>140.000mm</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2557,12 +2557,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>69.800mm</t>
+          <t>79.000mm</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>127.400mm</t>
+          <t>166.800mm</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -2584,12 +2584,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>21.000mm</t>
+          <t>7.000mm</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>73.500mm</t>
+          <t>91.500mm</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2611,12 +2611,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>27.000mm</t>
+          <t>13.000mm</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>75.000mm</t>
+          <t>93.000mm</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2638,12 +2638,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>21.500mm</t>
+          <t>7.500mm</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>65.500mm</t>
+          <t>83.500mm</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2665,12 +2665,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>26.000mm</t>
+          <t>12.000mm</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>58.500mm</t>
+          <t>76.500mm</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>93.000mm</t>
+          <t>104.500mm</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -2719,12 +2719,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>17.000mm</t>
+          <t>20.000mm</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>96.500mm</t>
+          <t>107.500mm</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2746,12 +2746,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>10.000mm</t>
+          <t>11.500mm</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>96.500mm</t>
+          <t>111.000mm</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
@@ -2773,12 +2773,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>22.000mm</t>
+          <t>25.000mm</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>105.500mm</t>
+          <t>116.500mm</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2800,12 +2800,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>28.000mm</t>
+          <t>31.000mm</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>105.500mm</t>
+          <t>116.500mm</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2827,12 +2827,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>32.500mm</t>
+          <t>35.500mm</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>105.500mm</t>
+          <t>116.500mm</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2854,12 +2854,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>36.500mm</t>
+          <t>39.500mm</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>96.500mm</t>
+          <t>107.500mm</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2881,12 +2881,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>44.000mm</t>
+          <t>47.000mm</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>96.500mm</t>
+          <t>107.500mm</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2908,12 +2908,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>46.500mm</t>
+          <t>49.500mm</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>93.500mm</t>
+          <t>104.500mm</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2935,12 +2935,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>46.000mm</t>
+          <t>49.000mm</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>89.000mm</t>
+          <t>100.000mm</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2962,12 +2962,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>36.000mm</t>
+          <t>39.000mm</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>84.000mm</t>
+          <t>91.500mm</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2989,12 +2989,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>49.000mm</t>
+          <t>52.000mm</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>83.500mm</t>
+          <t>91.000mm</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3016,12 +3016,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>58.000mm</t>
+          <t>65.000mm</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>94.500mm</t>
+          <t>92.500mm</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3043,12 +3043,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>72.500mm</t>
+          <t>79.500mm</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>90.000mm</t>
+          <t>88.000mm</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3070,12 +3070,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>69.800mm</t>
+          <t>79.000mm</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>72.400mm</t>
+          <t>114.800mm</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3085,7 +3085,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -3097,12 +3097,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>21.000mm</t>
+          <t>7.000mm</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>18.500mm</t>
+          <t>39.500mm</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3124,12 +3124,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>27.000mm</t>
+          <t>13.000mm</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>20.000mm</t>
+          <t>41.000mm</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -3151,12 +3151,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>21.500mm</t>
+          <t>7.500mm</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10.500mm</t>
+          <t>31.500mm</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -3178,12 +3178,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>26.000mm</t>
+          <t>12.000mm</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>3.500mm</t>
+          <t>24.500mm</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>38.000mm</t>
+          <t>52.500mm</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -3232,12 +3232,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>17.000mm</t>
+          <t>20.000mm</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>41.500mm</t>
+          <t>55.500mm</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -3259,12 +3259,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>10.000mm</t>
+          <t>11.500mm</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>41.500mm</t>
+          <t>59.000mm</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3274,7 +3274,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
     </row>
@@ -3286,12 +3286,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>22.000mm</t>
+          <t>25.000mm</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>50.500mm</t>
+          <t>64.500mm</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3313,12 +3313,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>28.000mm</t>
+          <t>31.000mm</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>50.500mm</t>
+          <t>64.500mm</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3340,12 +3340,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>32.500mm</t>
+          <t>35.500mm</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>50.500mm</t>
+          <t>64.500mm</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3367,12 +3367,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>36.500mm</t>
+          <t>39.500mm</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>41.500mm</t>
+          <t>55.500mm</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3394,12 +3394,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>44.000mm</t>
+          <t>47.000mm</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>41.500mm</t>
+          <t>55.500mm</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3421,12 +3421,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>46.500mm</t>
+          <t>49.500mm</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>38.500mm</t>
+          <t>52.500mm</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3448,12 +3448,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>46.000mm</t>
+          <t>49.000mm</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>34.000mm</t>
+          <t>48.000mm</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3475,12 +3475,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>36.000mm</t>
+          <t>39.000mm</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>29.000mm</t>
+          <t>39.500mm</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3502,12 +3502,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>49.000mm</t>
+          <t>52.000mm</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>28.500mm</t>
+          <t>39.000mm</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3529,12 +3529,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>58.000mm</t>
+          <t>65.000mm</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>39.500mm</t>
+          <t>40.500mm</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3556,12 +3556,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>72.500mm</t>
+          <t>79.500mm</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>35.000mm</t>
+          <t>36.000mm</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3583,12 +3583,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>69.800mm</t>
+          <t>79.000mm</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>17.400mm</t>
+          <t>62.800mm</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -3610,12 +3610,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>66.000mm</t>
+          <t>17.000mm</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>117.925mm</t>
+          <t>191.425mm</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>64.000mm</t>
+          <t>82.000mm</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>64.500mm</t>
+          <t>9.500mm</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3664,12 +3664,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>64.000mm</t>
+          <t>71.000mm</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>145.000mm</t>
+          <t>140.000mm</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -3691,12 +3691,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>68.190mm</t>
+          <t>73.190mm</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>132.240mm</t>
+          <t>165.240mm</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -3718,12 +3718,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>64.000mm</t>
+          <t>71.000mm</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>90.000mm</t>
+          <t>88.000mm</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -3745,12 +3745,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>68.190mm</t>
+          <t>73.190mm</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>77.240mm</t>
+          <t>113.240mm</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -3772,12 +3772,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>64.000mm</t>
+          <t>71.000mm</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>35.000mm</t>
+          <t>36.000mm</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -3799,12 +3799,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>68.190mm</t>
+          <t>73.190mm</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>22.240mm</t>
+          <t>61.240mm</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -3826,12 +3826,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>33.000mm</t>
+          <t>19.000mm</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>115.500mm</t>
+          <t>130.500mm</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -3853,12 +3853,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>43.000mm</t>
+          <t>46.000mm</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>134.000mm</t>
+          <t>138.500mm</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -3880,12 +3880,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>33.000mm</t>
+          <t>19.000mm</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>60.500mm</t>
+          <t>78.500mm</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -3907,12 +3907,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>43.000mm</t>
+          <t>46.000mm</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>79.000mm</t>
+          <t>86.500mm</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -3934,12 +3934,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>33.000mm</t>
+          <t>19.000mm</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>5.500mm</t>
+          <t>26.500mm</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -3961,12 +3961,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>43.000mm</t>
+          <t>46.000mm</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>24.000mm</t>
+          <t>34.500mm</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">

</xml_diff>

<commit_message>
Variante 3ch: disposizione piu' ordinata e fori di fissaggio M3
- scheda 103 x 215 mm: colonne distanziate (>= 2 mm tra i riquadri), spostamenti
  multipli della griglia del router
- serigrafia: riquadri della stessa riga con bordi allineati, titoli fissi,
  sottotitoli sotto il riquadro, frecce del segnale calcolate tra i blocchi,
  avviso 41 V nel blocco ALTA TENSIONE
- 8 fori M3 metallizzati a massa (angoli e confini tra i canali)
- routing rifatto: 0 errori DRC/connettivita', monitor a 1,6 mm dai nodi sensibili
- render, PDF, presentazione aggiornati

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fc9yPsNewCQrMK8R1c8Ls
</commit_message>
<xml_diff>
--- a/hardware/variante_3ch/jlcpcb/CPL_JLCPCB.xlsx
+++ b/hardware/variante_3ch/jlcpcb/CPL_JLCPCB.xlsx
@@ -451,12 +451,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>39.000mm</t>
+          <t>47.255mm</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>188.500mm</t>
+          <t>198.500mm</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -478,12 +478,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>44.500mm</t>
+          <t>52.755mm</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>198.000mm</t>
+          <t>208.000mm</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -505,12 +505,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>48.500mm</t>
+          <t>56.755mm</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>198.000mm</t>
+          <t>208.000mm</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -532,12 +532,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>29.000mm</t>
+          <t>37.255mm</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>201.000mm</t>
+          <t>211.000mm</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -559,12 +559,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>57.000mm</t>
+          <t>65.255mm</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>189.500mm</t>
+          <t>199.500mm</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>132.000mm</t>
+          <t>142.000mm</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>156.500mm</t>
+          <t>166.500mm</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -640,12 +640,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>16.500mm</t>
+          <t>18.405mm</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>164.000mm</t>
+          <t>174.000mm</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -667,12 +667,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>54.500mm</t>
+          <t>58.310mm</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>156.500mm</t>
+          <t>166.500mm</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -694,12 +694,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>43.500mm</t>
+          <t>47.310mm</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>164.000mm</t>
+          <t>174.000mm</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -721,12 +721,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>65.000mm</t>
+          <t>71.350mm</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>136.000mm</t>
+          <t>146.000mm</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>142.500mm</t>
+          <t>152.500mm</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>80.000mm</t>
+          <t>88.000mm</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>104.500mm</t>
+          <t>112.500mm</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -829,12 +829,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>16.500mm</t>
+          <t>18.405mm</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>112.000mm</t>
+          <t>120.000mm</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -856,12 +856,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>54.500mm</t>
+          <t>58.310mm</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>104.500mm</t>
+          <t>112.500mm</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -883,12 +883,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>43.500mm</t>
+          <t>47.310mm</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>112.000mm</t>
+          <t>120.000mm</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -910,12 +910,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>65.000mm</t>
+          <t>71.350mm</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>84.000mm</t>
+          <t>92.000mm</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>90.500mm</t>
+          <t>98.500mm</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>28.000mm</t>
+          <t>34.000mm</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>52.500mm</t>
+          <t>58.500mm</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1018,12 +1018,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>16.500mm</t>
+          <t>18.405mm</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>60.000mm</t>
+          <t>66.000mm</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1045,12 +1045,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>54.500mm</t>
+          <t>58.310mm</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>52.500mm</t>
+          <t>58.500mm</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1072,12 +1072,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>43.500mm</t>
+          <t>47.310mm</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>60.000mm</t>
+          <t>66.000mm</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1099,12 +1099,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>65.000mm</t>
+          <t>71.350mm</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>32.000mm</t>
+          <t>38.000mm</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>38.500mm</t>
+          <t>44.500mm</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1153,12 +1153,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>67.000mm</t>
+          <t>77.795mm</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>197.000mm</t>
+          <t>207.000mm</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1180,12 +1180,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>67.000mm</t>
+          <t>77.795mm</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>187.000mm</t>
+          <t>197.000mm</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1207,12 +1207,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>14.000mm</t>
+          <t>20.350mm</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>185.000mm</t>
+          <t>195.000mm</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1234,12 +1234,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>20.000mm</t>
+          <t>26.350mm</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>185.000mm</t>
+          <t>195.000mm</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1261,12 +1261,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>82.000mm</t>
+          <t>88.350mm</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14.500mm</t>
+          <t>18.500mm</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1288,12 +1288,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>77.000mm</t>
+          <t>89.535mm</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>201.000mm</t>
+          <t>193.000mm</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1315,12 +1315,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>27.500mm</t>
+          <t>29.405mm</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>171.500mm</t>
+          <t>181.500mm</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1342,12 +1342,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>54.500mm</t>
+          <t>58.310mm</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>169.000mm</t>
+          <t>179.000mm</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1369,12 +1369,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>76.000mm</t>
+          <t>82.350mm</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>145.000mm</t>
+          <t>155.000mm</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>65.500mm</t>
+          <t>71.850mm</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>140.000mm</t>
+          <t>150.000mm</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1423,12 +1423,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>73.000mm</t>
+          <t>79.350mm</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>170.000mm</t>
+          <t>180.000mm</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1450,12 +1450,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>27.500mm</t>
+          <t>29.405mm</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>119.500mm</t>
+          <t>127.500mm</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1477,12 +1477,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>54.500mm</t>
+          <t>58.310mm</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>117.000mm</t>
+          <t>125.000mm</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1504,12 +1504,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>76.000mm</t>
+          <t>82.350mm</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>93.000mm</t>
+          <t>101.000mm</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>65.500mm</t>
+          <t>71.850mm</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>88.000mm</t>
+          <t>96.000mm</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>73.000mm</t>
+          <t>79.350mm</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>118.000mm</t>
+          <t>126.000mm</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1585,12 +1585,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>27.500mm</t>
+          <t>29.405mm</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>67.500mm</t>
+          <t>73.500mm</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1612,12 +1612,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>54.500mm</t>
+          <t>58.310mm</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>65.000mm</t>
+          <t>71.000mm</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1639,12 +1639,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>76.000mm</t>
+          <t>82.350mm</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>41.000mm</t>
+          <t>47.000mm</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1666,12 +1666,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>65.500mm</t>
+          <t>71.850mm</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>36.000mm</t>
+          <t>42.000mm</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1693,12 +1693,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>73.000mm</t>
+          <t>79.350mm</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>66.000mm</t>
+          <t>72.000mm</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1720,12 +1720,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>79.500mm</t>
+          <t>85.850mm</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>134.000mm</t>
+          <t>144.000mm</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1747,12 +1747,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>79.500mm</t>
+          <t>85.850mm</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>82.000mm</t>
+          <t>90.000mm</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1774,12 +1774,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>79.500mm</t>
+          <t>85.850mm</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>30.000mm</t>
+          <t>36.000mm</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1801,12 +1801,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>31.000mm</t>
+          <t>39.255mm</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>194.000mm</t>
+          <t>204.000mm</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1828,12 +1828,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>25.000mm</t>
+          <t>26.905mm</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>162.117mm</t>
+          <t>172.117mm</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>35.500mm</t>
+          <t>37.405mm</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>163.383mm</t>
+          <t>173.383mm</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1882,12 +1882,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>25.000mm</t>
+          <t>26.905mm</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>110.117mm</t>
+          <t>118.117mm</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1909,12 +1909,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>35.500mm</t>
+          <t>37.405mm</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>111.383mm</t>
+          <t>119.383mm</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1936,12 +1936,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>25.000mm</t>
+          <t>26.905mm</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>58.117mm</t>
+          <t>64.117mm</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1963,12 +1963,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>35.500mm</t>
+          <t>37.405mm</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>59.383mm</t>
+          <t>65.383mm</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1990,12 +1990,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>49.500mm</t>
+          <t>57.755mm</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>188.000mm</t>
+          <t>198.000mm</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2017,12 +2017,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>46.500mm</t>
+          <t>54.755mm</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>188.000mm</t>
+          <t>198.000mm</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2044,12 +2044,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>39.000mm</t>
+          <t>47.255mm</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>192.000mm</t>
+          <t>202.000mm</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2071,12 +2071,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>43.500mm</t>
+          <t>51.755mm</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>188.000mm</t>
+          <t>198.000mm</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2098,12 +2098,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>85.500mm</t>
+          <t>91.850mm</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>8.500mm</t>
+          <t>12.500mm</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2125,12 +2125,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>61.200mm</t>
+          <t>67.550mm</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>13.000mm</t>
+          <t>17.000mm</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2152,12 +2152,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>67.200mm</t>
+          <t>73.550mm</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>13.000mm</t>
+          <t>17.000mm</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2179,12 +2179,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>73.200mm</t>
+          <t>79.550mm</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>13.000mm</t>
+          <t>17.000mm</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2206,12 +2206,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>57.000mm</t>
+          <t>65.255mm</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>200.000mm</t>
+          <t>210.000mm</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2233,12 +2233,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>57.000mm</t>
+          <t>65.255mm</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>194.500mm</t>
+          <t>204.500mm</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2260,12 +2260,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>87.300mm</t>
+          <t>96.600mm</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>195.000mm</t>
+          <t>200.000mm</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2287,12 +2287,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>87.300mm</t>
+          <t>96.600mm</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>192.000mm</t>
+          <t>197.000mm</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>143.500mm</t>
+          <t>153.500mm</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>145.000mm</t>
+          <t>155.000mm</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>135.500mm</t>
+          <t>145.500mm</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>128.500mm</t>
+          <t>138.500mm</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>156.500mm</t>
+          <t>166.500mm</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2449,12 +2449,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>20.000mm</t>
+          <t>21.905mm</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>159.500mm</t>
+          <t>169.500mm</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>163.000mm</t>
+          <t>173.000mm</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2503,12 +2503,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>25.000mm</t>
+          <t>26.905mm</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>168.500mm</t>
+          <t>178.500mm</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2530,12 +2530,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>31.000mm</t>
+          <t>32.905mm</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>168.500mm</t>
+          <t>178.500mm</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2557,12 +2557,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>35.500mm</t>
+          <t>37.405mm</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>168.500mm</t>
+          <t>178.500mm</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2584,12 +2584,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>39.500mm</t>
+          <t>41.405mm</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>159.500mm</t>
+          <t>169.500mm</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2611,12 +2611,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>47.000mm</t>
+          <t>50.810mm</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>159.500mm</t>
+          <t>169.500mm</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2638,12 +2638,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>49.500mm</t>
+          <t>53.310mm</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>156.500mm</t>
+          <t>166.500mm</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2665,12 +2665,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>49.000mm</t>
+          <t>52.810mm</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>152.000mm</t>
+          <t>162.000mm</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2692,12 +2692,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>39.000mm</t>
+          <t>42.810mm</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>143.500mm</t>
+          <t>153.500mm</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2719,12 +2719,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>52.000mm</t>
+          <t>55.810mm</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>143.000mm</t>
+          <t>153.000mm</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2746,12 +2746,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>65.000mm</t>
+          <t>71.350mm</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>144.500mm</t>
+          <t>154.500mm</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2773,12 +2773,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>79.500mm</t>
+          <t>85.850mm</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>140.000mm</t>
+          <t>150.000mm</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2800,12 +2800,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>79.000mm</t>
+          <t>85.350mm</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>166.800mm</t>
+          <t>176.800mm</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>145.000mm</t>
+          <t>155.000mm</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>142.500mm</t>
+          <t>152.500mm</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>91.500mm</t>
+          <t>99.500mm</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>93.000mm</t>
+          <t>101.000mm</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>83.500mm</t>
+          <t>91.500mm</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2967,7 +2967,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>76.500mm</t>
+          <t>84.500mm</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>104.500mm</t>
+          <t>112.500mm</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3016,12 +3016,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>20.000mm</t>
+          <t>21.905mm</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>107.500mm</t>
+          <t>115.500mm</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3048,7 +3048,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>111.000mm</t>
+          <t>119.000mm</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3070,12 +3070,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>25.000mm</t>
+          <t>26.905mm</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>116.500mm</t>
+          <t>124.500mm</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3097,12 +3097,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>31.000mm</t>
+          <t>32.905mm</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>116.500mm</t>
+          <t>124.500mm</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3124,12 +3124,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>35.500mm</t>
+          <t>37.405mm</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>116.500mm</t>
+          <t>124.500mm</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -3151,12 +3151,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>39.500mm</t>
+          <t>41.405mm</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>107.500mm</t>
+          <t>115.500mm</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -3178,12 +3178,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>47.000mm</t>
+          <t>50.810mm</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>107.500mm</t>
+          <t>115.500mm</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -3205,12 +3205,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>49.500mm</t>
+          <t>53.310mm</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>104.500mm</t>
+          <t>112.500mm</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -3232,12 +3232,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>49.000mm</t>
+          <t>52.810mm</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>100.000mm</t>
+          <t>108.000mm</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -3259,12 +3259,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>39.000mm</t>
+          <t>42.810mm</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>91.500mm</t>
+          <t>99.500mm</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3286,12 +3286,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>52.000mm</t>
+          <t>55.810mm</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>91.000mm</t>
+          <t>99.000mm</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3313,12 +3313,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>65.000mm</t>
+          <t>71.350mm</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>92.500mm</t>
+          <t>100.500mm</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3340,12 +3340,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>79.500mm</t>
+          <t>85.850mm</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>88.000mm</t>
+          <t>96.000mm</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3367,12 +3367,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>79.000mm</t>
+          <t>85.350mm</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>114.800mm</t>
+          <t>122.800mm</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3399,7 +3399,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>93.000mm</t>
+          <t>101.000mm</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>90.500mm</t>
+          <t>98.500mm</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>39.500mm</t>
+          <t>45.500mm</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>41.000mm</t>
+          <t>47.000mm</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>31.500mm</t>
+          <t>37.500mm</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>24.500mm</t>
+          <t>30.500mm</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>52.500mm</t>
+          <t>58.500mm</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3583,12 +3583,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>20.000mm</t>
+          <t>21.905mm</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>55.500mm</t>
+          <t>61.500mm</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>59.000mm</t>
+          <t>65.000mm</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>25.000mm</t>
+          <t>26.905mm</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>64.500mm</t>
+          <t>70.500mm</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3664,12 +3664,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>31.000mm</t>
+          <t>32.905mm</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>64.500mm</t>
+          <t>70.500mm</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -3691,12 +3691,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>35.500mm</t>
+          <t>37.405mm</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>64.500mm</t>
+          <t>70.500mm</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -3718,12 +3718,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>39.500mm</t>
+          <t>41.405mm</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>55.500mm</t>
+          <t>61.500mm</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -3745,12 +3745,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>47.000mm</t>
+          <t>50.810mm</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>55.500mm</t>
+          <t>61.500mm</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -3772,12 +3772,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>49.500mm</t>
+          <t>53.310mm</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>52.500mm</t>
+          <t>58.500mm</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -3799,12 +3799,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>49.000mm</t>
+          <t>52.810mm</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>48.000mm</t>
+          <t>54.000mm</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -3826,12 +3826,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>39.000mm</t>
+          <t>42.810mm</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>39.500mm</t>
+          <t>45.500mm</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -3853,12 +3853,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>52.000mm</t>
+          <t>55.810mm</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>39.000mm</t>
+          <t>45.000mm</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -3880,12 +3880,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>65.000mm</t>
+          <t>71.350mm</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>40.500mm</t>
+          <t>46.500mm</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -3907,12 +3907,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>79.500mm</t>
+          <t>85.850mm</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>36.000mm</t>
+          <t>42.000mm</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -3934,12 +3934,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>79.000mm</t>
+          <t>85.350mm</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>62.800mm</t>
+          <t>68.800mm</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -3966,7 +3966,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>41.000mm</t>
+          <t>47.000mm</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -3993,7 +3993,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>38.500mm</t>
+          <t>44.500mm</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -4015,12 +4015,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>17.000mm</t>
+          <t>23.350mm</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>191.425mm</t>
+          <t>201.425mm</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -4042,12 +4042,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>82.000mm</t>
+          <t>88.350mm</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>9.500mm</t>
+          <t>13.500mm</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -4069,12 +4069,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>79.500mm</t>
+          <t>89.535mm</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>194.000mm</t>
+          <t>199.500mm</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -4096,12 +4096,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>71.000mm</t>
+          <t>77.350mm</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>140.000mm</t>
+          <t>150.000mm</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -4123,12 +4123,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>73.190mm</t>
+          <t>79.540mm</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>165.240mm</t>
+          <t>175.240mm</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -4150,12 +4150,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>71.000mm</t>
+          <t>77.350mm</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>88.000mm</t>
+          <t>96.000mm</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -4177,12 +4177,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>73.190mm</t>
+          <t>79.540mm</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>113.240mm</t>
+          <t>121.240mm</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -4204,12 +4204,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>71.000mm</t>
+          <t>77.350mm</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>36.000mm</t>
+          <t>42.000mm</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -4231,12 +4231,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>73.190mm</t>
+          <t>79.540mm</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>61.240mm</t>
+          <t>67.240mm</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -4263,7 +4263,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>130.500mm</t>
+          <t>140.500mm</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -4285,12 +4285,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>46.000mm</t>
+          <t>49.810mm</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>138.500mm</t>
+          <t>148.500mm</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>78.500mm</t>
+          <t>86.500mm</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -4339,12 +4339,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>46.000mm</t>
+          <t>49.810mm</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>86.500mm</t>
+          <t>94.500mm</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>26.500mm</t>
+          <t>32.500mm</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -4393,12 +4393,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>46.000mm</t>
+          <t>49.810mm</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>34.500mm</t>
+          <t>40.500mm</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">

</xml_diff>